<commit_message>
Fixed meshing scheme. Changed from uniform meshing to meshing scheme defind by LGL points. Point force cases seem to be working.
</commit_message>
<xml_diff>
--- a/Verification.xlsx
+++ b/Verification.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kartikayshukla/Desktop/GRA/Models/FEM Models/Simo's static model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8405C175-F5CC-094B-ABFE-7BE2287FD6C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6236C38E-7900-4641-ABC9-FAB0CDAB3E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17200" xr2:uid="{399D07C8-64DA-784B-A3CF-75A5D5A1FD24}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{399D07C8-64DA-784B-A3CF-75A5D5A1FD24}"/>
   </bookViews>
   <sheets>
     <sheet name="Verification" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="152">
   <si>
     <t>SSB with Uniform load</t>
   </si>
@@ -502,14 +502,6 @@
         'Ry': [4*np.pi],
         'Rz': [0]
         }</t>
-  </si>
-  <si>
-    <t>NEL=100
-NNPEL=2
-DOFPN = 6
-NGQP = 1
-iterations = 10
-convergence = 1E-5</t>
   </si>
   <si>
     <t>Pure bending of cantilever beam about Y axis</t>
@@ -558,18 +550,6 @@
 Rotation about: X = 0, Y = -0.722789,, Z=0</t>
   </si>
   <si>
-    <t xml:space="preserve">13 iterations for E-5 convergence. </t>
-  </si>
-  <si>
-    <t>NEL=50
-NNPEL=2
-DOFPN = 6
-NGQP = 1
-iterations = 15
-convergence = 1E-8
-loadsteps = 2</t>
-  </si>
-  <si>
     <t>Deflection at Z=1m
 Translation: X = -0.0151964 m, Y=0, Z= 0.9998617 m
 Rotation about: X = 0, Y=-0.0228528186, Z=0</t>
@@ -689,15 +669,115 @@
     <t>Twist angle = TL/GJ = 1.1967966328888697*1/80E9*1.904761E-11 = np.pi/4 = 0.7853981633974483 rad = 45 deg</t>
   </si>
   <si>
+    <t>2 iterations for E-5 convergence.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">2 iterations for E-5 convergence. Since there are 10 full rotations, slope at Z=1m is 0 (or very close to it). See slope about Z axis plot for understanding the result. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>Expecting change in length but model results show no change because Poynting effect for steel is negligble - maximum change that can be expected is ~3-4mm. (how ? why?)
+https://en.wikipedia.org/wiki/Poynting_effect</t>
+    </r>
+  </si>
+  <si>
+    <t>NEL=100
+NNPEL=2
+DOFPN = 6
+NGQP=1
+iterations = 10
+convergence = 1E-5
+loadSteps = 10</t>
+  </si>
+  <si>
+    <t>Twist angle = TL/GJ = 95.74373063110957*1/80E9*1.904761E-11 = np.pi * 20= 3600 deg = 10 wraps
+Change in Length = delta L = k T^2L/G^2J^2 = k*95.74373063110957^2*1/( 80E9*1.904761E-11)^2 = 3947.841760435743 *k
+k for steel ranges from E-6 to E-8 so change in length = 0.03 to 3.947 mm</t>
+  </si>
+  <si>
     <t>Deflection at Z=1m
-Translation: X = 0 m, Y= 0 m, Z= 0
-Rotation about: X = 0.00743815 , Y= 0, Z= 0.7853981633974486 rad</t>
-  </si>
-  <si>
-    <t>2 iterations for E-5 convergence</t>
-  </si>
-  <si>
-    <t>Twist angle = TL/GJ = 95.74373063110957*1/80E9*1.904761E-11 = np.pi * 20= 3600 deg = 10 wraps</t>
+Translation: X = 0 m, Y= 0 m, Z= 1 m
+Rotation about: X = 0 , Y= 0, Z= 0.7853981633974486 rad</t>
+  </si>
+  <si>
+    <t>After rotNBC transformation</t>
+  </si>
+  <si>
+    <t>Deflection at Z=1m
+Translation: X = 0 m, Y= 0 m, Z= 1.000009523809524 m
+Rotation about: X = 0 , Y= 0, Z= 0</t>
+  </si>
+  <si>
+    <t>Deflection at Z=1m
+Translation: X = 0 m, Y= 0 m, Z=0.9999904761904761 m
+Rotation about: X = 0 , Y= 0, Z= 0</t>
+  </si>
+  <si>
+    <t>NEL=50
+NNPEL=2
+DOFPN = 6
+NGQP = 1
+iterations = 15
+convergence = 1E-5
+loadsteps = 2</t>
+  </si>
+  <si>
+    <t>Deflection at Z=1m
+Translation: X = 0 m, Y= 0.001289978199861985 m, Z= 0.02087442055911301 m
+Rotation about: X = 0.007434815095202058 rad , Y= 0, Z= 0
+Convergence in 4 iterations</t>
+  </si>
+  <si>
+    <t>Deflection at Z=1m
+Translation: X = -0.015198761457044163 m, Y=0, Z= 0.9998614868603563 m
+Rotation about: X = 0, Y= -0.022856752254535814 rad, Z=0</t>
+  </si>
+  <si>
+    <t>Deflection at Z=1m
+Translation: X = 0 m, Y= -0.015198761455870865 m, Z= 0.9998614868603833 m
+Rotation about: X = 0.022856752252697704 rad, Y= 0 , Z=0</t>
+  </si>
+  <si>
+    <t>Deflection at Z=1m
+Translation: X = -0.0012880944554900522 m, Y= 0 m, Z= 0.020874234375601864 m
+Rotation about: X = 0 , Y= 0.007489183566508229 rad, Z= 0
+Convergence in 4 iterations</t>
+  </si>
+  <si>
+    <t>Deflection at Z=1m
+Translation: X = -0.538194612555484 m, Y=0, Z= 0.7994733016199111 m
+Rotation about: X = 0, Y= -0.890396464901245 rad, Z=0
+8 iterations for first loadstep 4 iterations for second loadstep for convergence.</t>
+  </si>
+  <si>
+    <t>13 iterations for E-5 convergence. 
+How do you verify?</t>
+  </si>
+  <si>
+    <t>Deflection at Z=1m
+Translation: X = 0 m, Y= 0 m, Z= 1 m
+Rotation about: X = 0 , Y= 0, Z= 2.08532049693422e-12 rad</t>
+  </si>
+  <si>
+    <t>Deflection at Z=1m
+Translation: X = 0 m, Y= 0 m, Z= 0.9999999999999999 m
+Rotation about: X = 0 , Y= 0, Z= -3.2014517587696094e-15 rad</t>
+  </si>
+  <si>
+    <t>2 iteration for E-8 convergence per load step.æ
+Working for elements/nodes combination of 2/2, 2/3, 2/4, 2/6, 2/10, 10/2, 10/3, 10/4, 10/6, 10/10, 100/2, 100/3, 100/4, 100/6, 100/10, 1000/2, 1000/3, and 1000/4. Results same up to 14th decimal digit. 100/4 iteration case took 802 seconds to solve.</t>
+  </si>
+  <si>
+    <t>6 iterations for E-5 convergence.
+Working for elements/nodes combination of 2/2, 2/3, 10/2. Results similar within 1%.
+Full integration method not working - results not matching for even number of nodes with full integration. With reduced integration (by 1) results matching. Tested upto 10 nodes and point test of 15 nodes.
+Not working: 2/4.</t>
   </si>
 </sst>
 </file>
@@ -707,7 +787,7 @@
   <numFmts count="1">
     <numFmt numFmtId="179" formatCode="0.00000000000"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -763,6 +843,24 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow (Body)"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="7" tint="-0.249977111117893"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="7" tint="-0.249977111117893"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -808,7 +906,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -843,6 +941,39 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1178,11 +1309,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8118B9E2-6713-C649-B8C0-96D0E5033C84}">
-  <dimension ref="A1:M28"/>
+  <dimension ref="A1:N28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
-    <col min="2" max="2" width="23.83203125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="23.83203125" style="17" customWidth="1"/>
     <col min="3" max="3" width="12.1640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="62.1640625" style="1" customWidth="1"/>
     <col min="5" max="5" width="30.5" style="1" customWidth="1"/>
@@ -1192,15 +1323,16 @@
     <col min="9" max="9" width="29.1640625" style="3" customWidth="1"/>
     <col min="10" max="11" width="32.1640625" style="1" customWidth="1"/>
     <col min="12" max="12" width="10.83203125" style="1"/>
-    <col min="13" max="13" width="26.83203125" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="10.83203125" style="1"/>
+    <col min="13" max="13" width="26.83203125" style="19" customWidth="1"/>
+    <col min="14" max="14" width="32" style="1" customWidth="1"/>
+    <col min="15" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="3" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" s="3" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="17" t="s">
         <v>4</v>
       </c>
       <c r="C1" s="3" t="s">
@@ -1233,22 +1365,25 @@
       <c r="L1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="17" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" s="14" customFormat="1" ht="221" x14ac:dyDescent="0.2">
+      <c r="N1" s="3" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" s="14" customFormat="1" ht="221" x14ac:dyDescent="0.2">
       <c r="A2" s="14">
         <v>1</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="21" t="s">
         <v>35</v>
       </c>
       <c r="C2" s="14" t="s">
         <v>58</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E2" s="16" t="s">
         <v>17</v>
@@ -1260,65 +1395,71 @@
         <v>15</v>
       </c>
       <c r="H2" s="14" t="s">
-        <v>115</v>
+        <v>141</v>
       </c>
       <c r="I2" s="12" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="J2" s="14" t="s">
         <v>29</v>
       </c>
       <c r="K2" s="11" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="L2" s="15"/>
-      <c r="M2" s="14" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" s="14" customFormat="1" ht="187" x14ac:dyDescent="0.2">
-      <c r="A3" s="14">
+      <c r="M2" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="N2" s="15" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" s="23" customFormat="1" ht="255" x14ac:dyDescent="0.2">
+      <c r="A3" s="23">
         <v>2</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="D3" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="E3" s="16" t="s">
+      <c r="E3" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="G3" s="14" t="s">
+      <c r="G3" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="H3" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="I3" s="15" t="s">
-        <v>116</v>
-      </c>
-      <c r="J3" s="14" t="s">
+      <c r="H3" s="23" t="s">
+        <v>117</v>
+      </c>
+      <c r="I3" s="26" t="s">
+        <v>113</v>
+      </c>
+      <c r="J3" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="K3" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="M3" s="14" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" s="14" customFormat="1" ht="187" x14ac:dyDescent="0.2">
+      <c r="K3" s="23" t="s">
+        <v>106</v>
+      </c>
+      <c r="M3" s="27" t="s">
+        <v>151</v>
+      </c>
+      <c r="N3" s="26" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" s="14" customFormat="1" ht="187" x14ac:dyDescent="0.2">
       <c r="A4" s="14">
         <v>3</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="21" t="s">
         <v>36</v>
       </c>
       <c r="C4" s="14" t="s">
@@ -1337,141 +1478,150 @@
         <v>43</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="J4" s="14" t="s">
         <v>50</v>
       </c>
       <c r="K4" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="M4" s="14" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" ht="187" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
+        <v>106</v>
+      </c>
+      <c r="M4" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="N4" s="15" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" s="23" customFormat="1" ht="204" x14ac:dyDescent="0.2">
+      <c r="A5" s="23">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H5" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="I5" s="26" t="s">
         <v>109</v>
       </c>
-      <c r="I5" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="J5" s="1" t="s">
+      <c r="J5" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="K5" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="M5" s="1" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" ht="187" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
+      <c r="M5" s="27" t="s">
+        <v>150</v>
+      </c>
+      <c r="N5" s="26" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" s="23" customFormat="1" ht="187" x14ac:dyDescent="0.2">
+      <c r="A6" s="23">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="H6" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="I6" s="3" t="s">
+      <c r="H6" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="I6" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="J6" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="K6" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="M6" s="1" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" s="14" customFormat="1" ht="187" x14ac:dyDescent="0.2">
-      <c r="A7" s="14">
+      <c r="M6" s="27" t="s">
+        <v>111</v>
+      </c>
+      <c r="N6" s="26" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" s="11" customFormat="1" ht="187" x14ac:dyDescent="0.2">
+      <c r="A7" s="11">
         <v>6</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="D7" s="16" t="s">
+      <c r="C7" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="E7" s="16" t="s">
+      <c r="E7" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="G7" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="H7" s="14" t="s">
-        <v>121</v>
-      </c>
-      <c r="I7" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="J7" s="14" t="s">
+      <c r="H7" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="I7" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="J7" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="K7" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="M7" s="14" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" s="11" customFormat="1" ht="204" x14ac:dyDescent="0.2">
-      <c r="A8" s="14">
+      <c r="K7" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="M7" s="20" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" s="11" customFormat="1" ht="204" x14ac:dyDescent="0.2">
+      <c r="A8" s="11">
         <v>7</v>
       </c>
-      <c r="B8" s="15" t="s">
-        <v>105</v>
+      <c r="B8" s="22" t="s">
+        <v>104</v>
       </c>
       <c r="C8" s="14" t="s">
         <v>58</v>
@@ -1489,21 +1639,24 @@
         <v>103</v>
       </c>
       <c r="H8" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="I8" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="M8" s="20" t="s">
+        <v>122</v>
+      </c>
+      <c r="N8" s="15" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="204" x14ac:dyDescent="0.2">
+      <c r="A9" s="11">
+        <v>8</v>
+      </c>
+      <c r="B9" s="22" t="s">
         <v>124</v>
-      </c>
-      <c r="I8" s="12" t="s">
-        <v>126</v>
-      </c>
-      <c r="M8" s="11" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" ht="204" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
-        <v>8</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>127</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>58</v>
@@ -1518,88 +1671,104 @@
         <v>32</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="H9" s="14" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I9" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="M9" s="20" t="s">
+        <v>126</v>
+      </c>
+      <c r="N9" s="15" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" s="23" customFormat="1" ht="204" x14ac:dyDescent="0.2">
+      <c r="A10" s="23">
+        <v>9</v>
+      </c>
+      <c r="B10" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="E10" s="25" t="s">
+        <v>97</v>
+      </c>
+      <c r="F10" s="23" t="s">
+        <v>32</v>
+      </c>
+      <c r="G10" s="23" t="s">
         <v>130</v>
       </c>
-      <c r="M9" s="11" t="s">
+      <c r="H10" s="23" t="s">
+        <v>131</v>
+      </c>
+      <c r="I10" s="26" t="s">
+        <v>137</v>
+      </c>
+      <c r="K10" s="23" t="s">
+        <v>132</v>
+      </c>
+      <c r="M10" s="27" t="s">
+        <v>133</v>
+      </c>
+      <c r="N10" s="26" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" s="11" customFormat="1" ht="238" x14ac:dyDescent="0.2">
+      <c r="A11" s="14">
+        <v>10</v>
+      </c>
+      <c r="B11" s="21" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" s="14" customFormat="1" ht="204" x14ac:dyDescent="0.2">
-      <c r="A10" s="14">
-        <v>9</v>
-      </c>
-      <c r="B10" s="15" t="s">
-        <v>132</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" s="16" t="s">
+      <c r="C11" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" s="16" t="s">
         <v>102</v>
       </c>
-      <c r="E10" s="16" t="s">
+      <c r="E11" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="F11" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="G10" s="14" t="s">
-        <v>133</v>
-      </c>
-      <c r="H10" s="14" t="s">
+      <c r="G11" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="H11" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="I11" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="J11" s="14"/>
+      <c r="K11" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="M11" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="I10" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="K10" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="M10" s="14" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" s="11" customFormat="1" ht="204" x14ac:dyDescent="0.2">
-      <c r="A11" s="11">
-        <v>10</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C11" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="D11" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E11" s="13" t="s">
-        <v>97</v>
-      </c>
-      <c r="F11" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="G11" s="11" t="s">
-        <v>133</v>
-      </c>
-      <c r="H11" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="I11" s="12" t="s">
-        <v>136</v>
-      </c>
-      <c r="K11" s="14" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" s="11" customFormat="1" ht="204" x14ac:dyDescent="0.2">
-      <c r="B12" s="12" t="s">
-        <v>106</v>
+      <c r="N11" s="15" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" s="11" customFormat="1" ht="204" x14ac:dyDescent="0.2">
+      <c r="A12" s="11">
+        <v>11</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>105</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>58</v>
@@ -1614,62 +1783,55 @@
         <v>32</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="H12" s="11" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I12" s="12"/>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="M12" s="20"/>
+    </row>
+    <row r="13" spans="1:14" s="11" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A13" s="11">
+        <v>12</v>
+      </c>
+      <c r="B13" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="I13" s="12"/>
+      <c r="M13" s="20"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:13" ht="204" x14ac:dyDescent="0.2">
-      <c r="B15" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="M15" s="1" t="s">
+    <row r="15" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="M15" s="19" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="55" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="16" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="19" spans="2:3" ht="52" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="17" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="17" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="21" spans="2:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="17" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="24" spans="2:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="17" t="s">
         <v>0</v>
       </c>
       <c r="C24" s="1" t="s">
@@ -1677,15 +1839,12 @@
       </c>
     </row>
     <row r="26" spans="2:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="B26" s="3" t="s">
-        <v>1</v>
-      </c>
       <c r="C26" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="27" spans="2:3" ht="51" x14ac:dyDescent="0.2">
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="17" t="s">
         <v>2</v>
       </c>
       <c r="C27" s="1" t="s">
@@ -1693,7 +1852,7 @@
       </c>
     </row>
     <row r="28" spans="2:3" ht="51" x14ac:dyDescent="0.2">
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="17" t="s">
         <v>9</v>
       </c>
       <c r="C28" s="1" t="s">
@@ -1714,7 +1873,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>